<commit_message>
adding chart of quickSelect
</commit_message>
<xml_diff>
--- a/week4/programming/quickSelect/Complexity_Chart.xlsx
+++ b/week4/programming/quickSelect/Complexity_Chart.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Work\UCA\week4\programming\quickSelect\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F60D79-E7CA-40E9-A5FB-C36D2DC68F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B246D7CF-BFD7-406E-B3E5-97A48F802714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Runtime Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Runtime Chart" sheetId="2" r:id="rId2"/>
+    <sheet name="Runtime Chart" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -193,66 +193,60 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Runtime Data'!$A$2:$A$9</c:f>
+              <c:f>'Runtime Data'!$A$2:$A$8</c:f>
               <c:numCache>
                 <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>10000</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>20000</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>40000</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>80000</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>160000</c:v>
-                </c:pt>
                 <c:pt idx="5">
-                  <c:v>320000</c:v>
+                  <c:v>12000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>640000</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1000000</c:v>
+                  <c:v>14000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Runtime Data'!$B$2:$B$9</c:f>
+              <c:f>'Runtime Data'!$B$2:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>6.6000000000000003E-2</c:v>
+                  <c:v>2.1999999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.104</c:v>
+                  <c:v>5.8000000000000003E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.46700000000000003</c:v>
+                  <c:v>4.7E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.78500000000000003</c:v>
+                  <c:v>7.9000000000000001E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.214</c:v>
+                  <c:v>0.111</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.4009999999999998</c:v>
+                  <c:v>0.161</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.9470000000000001</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>8.4380000000000006</c:v>
+                  <c:v>0.122</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -260,7 +254,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9776-4813-968A-69495971F431}"/>
+              <c16:uniqueId val="{00000001-704B-4F79-A61B-05F5E4303632}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -274,11 +268,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="1281357327"/>
-        <c:axId val="1280792879"/>
+        <c:axId val="411030048"/>
+        <c:axId val="341098800"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1281357327"/>
+        <c:axId val="411030048"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -307,7 +301,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1280792879"/>
+        <c:crossAx val="341098800"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -315,7 +309,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1280792879"/>
+        <c:axId val="341098800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -344,7 +338,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1281357327"/>
+        <c:crossAx val="411030048"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -388,7 +382,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E23A005F-A879-BFD4-6559-9319507BFB11}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4F8B1B0-0F89-299F-20B8-53DB9ED367B0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -706,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -723,66 +717,58 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="B2" s="3">
-        <v>6.6000000000000003E-2</v>
+        <v>2.1999999999999999E-2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="B3" s="3">
-        <v>0.104</v>
+        <v>5.8000000000000003E-2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>40000</v>
+        <v>6000</v>
       </c>
       <c r="B4" s="3">
-        <v>0.46700000000000003</v>
+        <v>4.7E-2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>80000</v>
+        <v>8000</v>
       </c>
       <c r="B5" s="3">
-        <v>0.78500000000000003</v>
+        <v>7.9000000000000001E-2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>160000</v>
+        <v>10000</v>
       </c>
       <c r="B6" s="3">
-        <v>2.214</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>320000</v>
+        <v>12000</v>
       </c>
       <c r="B7" s="3">
-        <v>5.4009999999999998</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>640000</v>
+        <v>14000</v>
       </c>
       <c r="B8" s="3">
-        <v>3.9470000000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>1000000</v>
-      </c>
-      <c r="B9" s="3">
-        <v>8.4380000000000006</v>
+        <v>0.122</v>
       </c>
     </row>
   </sheetData>
@@ -791,7 +777,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41938674-0C6F-4298-A46F-6EBFFEE65B68}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B246F7-AFAA-4721-A6C4-90B27EEA09A6}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>